<commit_message>
Added Retry mechanism for step.
On every Step atleast 3 seconds would be spent.
If step fails in lesser than 3 seconds then retry it.
</commit_message>
<xml_diff>
--- a/TestPlan.xlsx
+++ b/TestPlan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gurcharan/Desktop/CouchBase/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4804731-512F-C745-814E-912B10BF08B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F56A1A-7CC3-2841-97B8-72067BCD9AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17680" xr2:uid="{83599564-6E6F-6145-9A4F-0A399FCEBD48}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="17680" xr2:uid="{83599564-6E6F-6145-9A4F-0A399FCEBD48}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="55">
   <si>
     <t>Sno</t>
   </si>
@@ -192,6 +192,15 @@
   </si>
   <si>
     <t>@allPages, @ProductPage</t>
+  </si>
+  <si>
+    <t>@allPages, @DownloadsPage, @DownloadsPageServerTab</t>
+  </si>
+  <si>
+    <t>@allPages, @DownloadsPage, @DownloadsPageKubernetesOperatorTab</t>
+  </si>
+  <si>
+    <t>@allPages, @DownloadsPage, @DownloadsPageMobileAndEdgeTab</t>
   </si>
 </sst>
 </file>
@@ -706,7 +715,7 @@
         <v>39</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -723,7 +732,7 @@
         <v>39</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -740,7 +749,7 @@
         <v>39</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>